<commit_message>
docs: publish approved full symbol and unit reference
</commit_message>
<xml_diff>
--- a/기호정리/symbols.xlsx
+++ b/기호정리/symbols.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기호" sheetId="1" r:id="R04b96eaee9804095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입력근거" sheetId="2" r:id="R42cce0028fcb4e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기호" sheetId="1" r:id="Rff0040ccdf3d472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입력근거" sheetId="2" r:id="Rf5bd5d49f0a147de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -134,8 +134,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnifiedSymbols" displayName="UnifiedSymbols" ref="A1:H49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H49"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnifiedSymbols" displayName="UnifiedSymbols" ref="A1:H60" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H60"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="분류"/>
     <x:tableColumn id="2" name="통일 기호"/>
@@ -151,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="InputEvidence" displayName="InputEvidence" ref="A1:H36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H36"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="InputEvidence" displayName="InputEvidence" ref="A1:H39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H39"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="범위"/>
     <x:tableColumn id="2" name="입력"/>
@@ -694,7 +694,7 @@
         <x:v>https://github.com/donghyeok8649daniel/al-fatigue-probability-theory/blob/c8ccff7553cbb2e66b0c37a76ee8a24808478824/README.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="60" customHeight="1">
+    <x:row r="11" ht="52" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>하중</x:v>
       </x:c>
@@ -718,6 +718,12 @@
       </x:c>
       <x:c r="H11" s="3" t="str">
         <x:v>S3 S8</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+      <x:c r="K11" s="9" t="str">
+        <x:v>기호정리/README.md의 분석 보조 명명 계약; production 채택 아님</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
@@ -1661,22 +1667,22 @@
         <x:v>기하</x:v>
       </x:c>
       <x:c r="B48" s="3" t="str">
-        <x:v>A_int</x:v>
+        <x:v>V_eff</x:v>
       </x:c>
       <x:c r="C48" s="3" t="str">
-        <x:v>같은 계면 대표계의 실제 면적</x:v>
+        <x:v>축 일 정합을 요구한 조건부 정규화 부피</x:v>
       </x:c>
       <x:c r="D48" s="3" t="str">
         <x:v>해당 없음</x:v>
       </x:c>
       <x:c r="E48" s="3" t="str">
-        <x:v>m²</x:v>
+        <x:v>m³</x:v>
       </x:c>
       <x:c r="F48" s="3" t="str">
-        <x:v>에너지 per-interface 정규화와 결속</x:v>
+        <x:v>측정 V_geom의 대체값 아님</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
-        <x:v>interface area</x:v>
+        <x:v>effective axial work volume</x:v>
       </x:c>
       <x:c r="H48" s="3" t="str">
         <x:v>S8</x:v>
@@ -1684,13 +1690,13 @@
     </x:row>
     <x:row r="49" ht="60" customHeight="1">
       <x:c r="A49" s="3" t="str">
-        <x:v>통계</x:v>
+        <x:v>기하</x:v>
       </x:c>
       <x:c r="B49" s="3" t="str">
-        <x:v>A_c</x:v>
+        <x:v>A_int</x:v>
       </x:c>
       <x:c r="C49" s="3" t="str">
-        <x:v>외부 보정된 상관 면적</x:v>
+        <x:v>같은 계면 대표계의 실제 면적</x:v>
       </x:c>
       <x:c r="D49" s="3" t="str">
         <x:v>해당 없음</x:v>
@@ -1699,19 +1705,305 @@
         <x:v>m²</x:v>
       </x:c>
       <x:c r="F49" s="3" t="str">
+        <x:v>에너지 per-interface 정규화와 결속</x:v>
+      </x:c>
+      <x:c r="G49" s="3" t="str">
+        <x:v>interface area</x:v>
+      </x:c>
+      <x:c r="H49" s="3" t="str">
+        <x:v>S8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="60" customHeight="1">
+      <x:c r="A50" s="3" t="str">
+        <x:v>통계</x:v>
+      </x:c>
+      <x:c r="B50" s="3" t="str">
+        <x:v>A_c</x:v>
+      </x:c>
+      <x:c r="C50" s="3" t="str">
+        <x:v>외부 보정된 상관 면적</x:v>
+      </x:c>
+      <x:c r="D50" s="3" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="E50" s="3" t="str">
+        <x:v>m²</x:v>
+      </x:c>
+      <x:c r="F50" s="3" t="str">
         <x:v>A_int/원자면적/FVM 면적과 등치 금지</x:v>
       </x:c>
-      <x:c r="G49" s="3" t="str">
+      <x:c r="G50" s="3" t="str">
         <x:v>correlation_area</x:v>
       </x:c>
-      <x:c r="H49" s="3" t="str">
+      <x:c r="H50" s="3" t="str">
         <x:v>S4 S8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="60" customHeight="1">
+      <x:c r="A51" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B51" s="3" t="str">
+        <x:v>P_hat_k / R_hat_k</x:v>
+      </x:c>
+      <x:c r="C51" s="3" t="str">
+        <x:v>positive raw-bin의 P / full-r 조건부 measure</x:v>
+      </x:c>
+      <x:c r="D51" s="3" t="str">
+        <x:v>확률 measure</x:v>
+      </x:c>
+      <x:c r="E51" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F51" s="3" t="str">
+        <x:v>P_hat은 p_k&gt;0; reference는 full bin 유지</x:v>
+      </x:c>
+      <x:c r="G51" s="3" t="str">
+        <x:v>conditional P_i,R_i</x:v>
+      </x:c>
+      <x:c r="H51" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="60" customHeight="1">
+      <x:c r="A52" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="str">
+        <x:v>alpha1^P,alpha2^P,gamma^P</x:v>
+      </x:c>
+      <x:c r="C52" s="3" t="str">
+        <x:v>P 조건부 두 mask marginals와 joint</x:v>
+      </x:c>
+      <x:c r="D52" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E52" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F52" s="3" t="str">
+        <x:v>R fractions로 기호만 바꾸어 대입 금지</x:v>
+      </x:c>
+      <x:c r="G52" s="3" t="str">
+        <x:v>SB21 alpha,beta,gamma</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="60" customHeight="1">
+      <x:c r="A53" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B53" s="3" t="str">
+        <x:v>beta1^R,beta2^R,beta12^R</x:v>
+      </x:c>
+      <x:c r="C53" s="3" t="str">
+        <x:v>R 조건부 marginals와 joint</x:v>
+      </x:c>
+      <x:c r="D53" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E53" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F53" s="3" t="str">
+        <x:v>missing joint를 product/0으로 채우지 않음</x:v>
+      </x:c>
+      <x:c r="G53" s="3" t="str">
+        <x:v>E20/E21 reference beta</x:v>
+      </x:c>
+      <x:c r="H53" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="60" customHeight="1">
+      <x:c r="A54" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B54" s="3" t="str">
+        <x:v>eta_P</x:v>
+      </x:c>
+      <x:c r="C54" s="3" t="str">
+        <x:v>gamma^P-alpha1^P alpha2^P</x:v>
+      </x:c>
+      <x:c r="D54" s="3" t="str">
+        <x:v>signed 1</x:v>
+      </x:c>
+      <x:c r="E54" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F54" s="3" t="str">
+        <x:v>reference c_R 및 energy budget eta_E와 구별</x:v>
+      </x:c>
+      <x:c r="G54" s="3" t="str">
+        <x:v>SB21 eta</x:v>
+      </x:c>
+      <x:c r="H54" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="60" customHeight="1">
+      <x:c r="A55" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B55" s="3" t="str">
+        <x:v>c_R</x:v>
+      </x:c>
+      <x:c r="C55" s="3" t="str">
+        <x:v>beta12^R-beta1^R beta2^R</x:v>
+      </x:c>
+      <x:c r="D55" s="3" t="str">
+        <x:v>signed 1</x:v>
+      </x:c>
+      <x:c r="E55" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F55" s="3" t="str">
+        <x:v>actual overlap volume가 아님</x:v>
+      </x:c>
+      <x:c r="G55" s="3" t="str">
+        <x:v>E21 cR</x:v>
+      </x:c>
+      <x:c r="H55" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="60" customHeight="1">
+      <x:c r="A56" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B56" s="3" t="str">
+        <x:v>D_KL,pre</x:v>
+      </x:c>
+      <x:c r="C56" s="3" t="str">
+        <x:v>sum p_k KL(P_hat_k||R_hat_k)</x:v>
+      </x:c>
+      <x:c r="D56" s="3" t="str">
+        <x:v>raw-weighted entropy</x:v>
+      </x:c>
+      <x:c r="E56" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F56" s="3" t="str">
+        <x:v>Gibbs/post/removed KL 및 diffusion D_i와 구별</x:v>
+      </x:c>
+      <x:c r="G56" s="3" t="str">
+        <x:v>E20/E21 D</x:v>
+      </x:c>
+      <x:c r="H56" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="60" customHeight="1">
+      <x:c r="A57" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B57" s="3" t="str">
+        <x:v>nu_F,k</x:v>
+      </x:c>
+      <x:c r="C57" s="3" t="str">
+        <x:v>full bin reference 질량 int_Bk r dq</x:v>
+      </x:c>
+      <x:c r="D57" s="3" t="str">
+        <x:v>reference mass</x:v>
+      </x:c>
+      <x:c r="E57" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F57" s="3" t="str">
+        <x:v>nu_B,stationary mass와 자동 등치 금지</x:v>
+      </x:c>
+      <x:c r="G57" s="3" t="str">
+        <x:v>nu_F,nu_i</x:v>
+      </x:c>
+      <x:c r="H57" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="60" customHeight="1">
+      <x:c r="A58" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B58" s="3" t="str">
+        <x:v>F_nu(p)</x:v>
+      </x:c>
+      <x:c r="C58" s="3" t="str">
+        <x:v>같은 g_k/theta/nu_F의 raw functional</x:v>
+      </x:c>
+      <x:c r="D58" s="3" t="str">
+        <x:v>raw-weighted energy</x:v>
+      </x:c>
+      <x:c r="E58" s="3" t="str">
+        <x:v>J (physical bridge 조건)</x:v>
+      </x:c>
+      <x:c r="F58" s="3" t="str">
+        <x:v>signed mass defect를 entropy state로 넣지 않음</x:v>
+      </x:c>
+      <x:c r="G58" s="3" t="str">
+        <x:v>F_bin</x:v>
+      </x:c>
+      <x:c r="H58" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="60" customHeight="1">
+      <x:c r="A59" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B59" s="3" t="str">
+        <x:v>eta_E, B_E</x:v>
+      </x:c>
+      <x:c r="C59" s="3" t="str">
+        <x:v>독립적으로 공급되는 절댓값 에너지 예산</x:v>
+      </x:c>
+      <x:c r="D59" s="3" t="str">
+        <x:v>raw-weighted energy</x:v>
+      </x:c>
+      <x:c r="E59" s="3" t="str">
+        <x:v>J (physical bridge 조건)</x:v>
+      </x:c>
+      <x:c r="F59" s="3" t="str">
+        <x:v>eta_P와 구별; scalar equality로 생성하지 않음</x:v>
+      </x:c>
+      <x:c r="G59" s="3" t="str">
+        <x:v>E20 eta,B</x:v>
+      </x:c>
+      <x:c r="H59" s="3" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="60" customHeight="1">
+      <x:c r="A60" s="3" t="str">
+        <x:v>분석보조</x:v>
+      </x:c>
+      <x:c r="B60" s="3" t="str">
+        <x:v>E_event, E_prod, C_R, C_F, B_KL</x:v>
+      </x:c>
+      <x:c r="C60" s="3" t="str">
+        <x:v>사건 오차/overlap/상한의 raw 질량</x:v>
+      </x:c>
+      <x:c r="D60" s="3" t="str">
+        <x:v>raw mass</x:v>
+      </x:c>
+      <x:c r="E60" s="3" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F60" s="3" t="str">
+        <x:v>상한을 actual overlap이나 lower bound로 대체 금지</x:v>
+      </x:c>
+      <x:c r="G60" s="3" t="str">
+        <x:v>E_M,E_prod,C_R,C_F,B_D</x:v>
+      </x:c>
+      <x:c r="H60" s="3" t="str">
+        <x:v>연구 정의</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20c85abcb87e4b82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d275a73ecc44ef2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1787,7 +2079,7 @@
         <x:v>N=1 UI 기준</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J2" s="9" t="str">
         <x:v>S1</x:v>
@@ -1819,7 +2111,7 @@
         <x:v>상속된 native 기준</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J3" s="9" t="str">
         <x:v>S2</x:v>
@@ -1851,7 +2143,7 @@
         <x:v>상속된 native 기준</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
         <x:v>S3</x:v>
@@ -1883,7 +2175,7 @@
         <x:v>상속된 native 기준</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
         <x:v>S4</x:v>
@@ -1915,7 +2207,7 @@
         <x:v>native thermal energy</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
         <x:v>S5</x:v>
@@ -1947,7 +2239,7 @@
         <x:v>native mobility</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
         <x:v>S6</x:v>
@@ -1979,7 +2271,7 @@
         <x:v>native mobility</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
         <x:v>S7</x:v>
@@ -2011,7 +2303,7 @@
         <x:v>기하 보정값 아님</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
         <x:v>S8</x:v>
@@ -2043,7 +2335,7 @@
         <x:v>기록된 역사적 기준; 재계산하지 않음</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
         <x:v>S9</x:v>
@@ -2052,7 +2344,7 @@
         <x:v>https://github.com/donghyeok8649daniel/al-fatigue-probability-theory/blob/c8ccff7553cbb2e66b0c37a76ee8a24808478824/README.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="60" customHeight="1">
+    <x:row r="11" ht="52" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>canonical_n1</x:v>
       </x:c>
@@ -2075,7 +2367,13 @@
         <x:v>같은 chi=.2 기준; 재계산하지 않음</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
+      </x:c>
+      <x:c r="J11" s="9" t="str">
+        <x:v>연구 정의</x:v>
+      </x:c>
+      <x:c r="K11" s="9" t="str">
+        <x:v>기호정리/README.md의 분석 보조 명명 계약; production 채택 아님</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
@@ -2101,7 +2399,7 @@
         <x:v>N1 프로파일과 별도</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
@@ -2127,7 +2425,7 @@
         <x:v>N1 프로파일과 별도</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -2153,7 +2451,7 @@
         <x:v>N1 프로파일과 별도</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
@@ -2179,7 +2477,7 @@
         <x:v>N1 프로파일과 별도</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
@@ -2205,7 +2503,7 @@
         <x:v>해당 FCC/eV reference 선언; 실제 결합 선택 아님</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
@@ -2231,7 +2529,7 @@
         <x:v>1 eV 단위 선언; kinetic 보정 아님</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -2257,7 +2555,7 @@
         <x:v>실제 선택된 run grid는 미정</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -2283,7 +2581,7 @@
         <x:v>실제 선택된 run grid는 미정</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -2309,7 +2607,7 @@
         <x:v>실제 step은 CFL에 의해 제한됨</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -2335,7 +2633,7 @@
         <x:v>기존 코드의 수치 제어값</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>기존 공개 source</x:v>
+        <x:v>기존 source</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -2353,13 +2651,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F22" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
         <x:v>같은 모형 ID·parameter fingerprint·per-atom/cell/interface counting과 채택 근거</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -2377,13 +2675,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F23" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
         <x:v>같은 좌표의 측정 길이·기준 lattice/상태·단위와 대응식</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
@@ -2401,13 +2699,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F24" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
         <x:v>같은 대표계 에너지·thermal normalization·보정 근거</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
@@ -2425,13 +2723,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F25" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
         <x:v>3D primitive vectors 또는 원자 좌표, 경계·두께·partition·집단 지지영역</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
@@ -2449,13 +2747,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F26" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
         <x:v>위 3D 자료와 동일한 대표계/기준 또는 현재 상태의 부피 측정</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -2473,13 +2771,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F27" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
         <x:v>계면의 두 접벡터 또는 동일 영역의 면적/법선·방위</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -2497,13 +2795,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
         <x:v>좌표 jump→strain의 orientation/기하, 공액 stress·strain·volume convention</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -2521,13 +2819,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F29" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
         <x:v>같은 소재·온도·방위·상태의 modulus와 측정/보정 원자료</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -2545,13 +2843,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F30" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
         <x:v>같은 specimen/MD record의 온도 로그 및 thermostat/ensemble</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
@@ -2569,13 +2867,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
         <x:v>같은 집단좌표·PMF·열항의 signed response 또는 covariance/확산 원자료, 오차와 coarse-time 검증</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
@@ -2593,13 +2891,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F32" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G32" s="3" t="str">
         <x:v>controller raw trace, 센서 단위/교정, cycle-to-stage map·sampling clock</x:v>
       </x:c>
       <x:c r="H32" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="60" customHeight="1">
@@ -2617,13 +2915,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F33" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G33" s="3" t="str">
         <x:v>초기 준비·선별·support, 실제 grid와 quadrature, preload·초기 absorber 기록</x:v>
       </x:c>
       <x:c r="H33" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
@@ -2641,13 +2939,13 @@
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F34" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
         <x:v>동일 stage의 원래 mask/geometry, 검사 last-negative/first-positive, 검출한계와 DCPD 교정</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="60" customHeight="1">
@@ -2655,23 +2953,23 @@
         <x:v>actual_coupled</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
-        <x:v>실제 상관 영역·집단 법칙</x:v>
+        <x:v>분석 reference의 형태와 full bin 질량</x:v>
       </x:c>
       <x:c r="C35" s="11"/>
       <x:c r="D35" s="3" t="str">
-        <x:v>m^2; joint law</x:v>
+        <x:v>reference mass</x:v>
       </x:c>
       <x:c r="E35" s="3" t="str">
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F35" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
-        <x:v>동일 하중/조직의 공간 위치·correlation/공동 사건 자료; 독립성 검증</x:v>
+        <x:v>고정 r(q), 동일 bin 적분·full nu_F·선택 이유; Gibbs 대체 여부 명시</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="60" customHeight="1">
@@ -2679,32 +2977,104 @@
         <x:v>actual_coupled</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
-        <x:v>실제 quadrature/runtime/source 오차</x:v>
+        <x:v>같은 P/R의 두 mask joint/overlap</x:v>
       </x:c>
       <x:c r="C36" s="11"/>
       <x:c r="D36" s="3" t="str">
-        <x:v>해당량 단위</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E36" s="3" t="str">
         <x:v>미정</x:v>
       </x:c>
       <x:c r="F36" s="3" t="str">
-        <x:v>S4 S8</x:v>
+        <x:v>필요 원자료</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
+        <x:v>동일 raw cohort·reference의 masks/joint integrals와 무중간변화 stage 근거</x:v>
+      </x:c>
+      <x:c r="H36" s="3" t="str">
+        <x:v>미확보/미결속</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="60" customHeight="1">
+      <x:c r="A37" s="3" t="str">
+        <x:v>actual_coupled</x:v>
+      </x:c>
+      <x:c r="B37" s="3" t="str">
+        <x:v>실제 pre KL·독립 energy/error budgets</x:v>
+      </x:c>
+      <x:c r="C37" s="11"/>
+      <x:c r="D37" s="3" t="str">
+        <x:v>entropy; J</x:v>
+      </x:c>
+      <x:c r="E37" s="3" t="str">
+        <x:v>미정</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
+        <x:v>필요 원자료</x:v>
+      </x:c>
+      <x:c r="G37" s="3" t="str">
+        <x:v>rho/r/reconstruction, proper finite functional 차이와 독립 절댓값 bound certificate</x:v>
+      </x:c>
+      <x:c r="H37" s="3" t="str">
+        <x:v>미확보/미결속</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="60" customHeight="1">
+      <x:c r="A38" s="3" t="str">
+        <x:v>actual_coupled</x:v>
+      </x:c>
+      <x:c r="B38" s="3" t="str">
+        <x:v>실제 상관 영역·집단 법칙</x:v>
+      </x:c>
+      <x:c r="C38" s="11"/>
+      <x:c r="D38" s="3" t="str">
+        <x:v>m^2; joint law</x:v>
+      </x:c>
+      <x:c r="E38" s="3" t="str">
+        <x:v>미정</x:v>
+      </x:c>
+      <x:c r="F38" s="3" t="str">
+        <x:v>필요 원자료</x:v>
+      </x:c>
+      <x:c r="G38" s="3" t="str">
+        <x:v>동일 하중/조직의 공간 위치·correlation/공동 사건 자료; 독립성 검증</x:v>
+      </x:c>
+      <x:c r="H38" s="3" t="str">
+        <x:v>미확보/미결속</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="60" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>actual_coupled</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="str">
+        <x:v>실제 quadrature/runtime/source 오차</x:v>
+      </x:c>
+      <x:c r="C39" s="11"/>
+      <x:c r="D39" s="3" t="str">
+        <x:v>해당량 단위</x:v>
+      </x:c>
+      <x:c r="E39" s="3" t="str">
+        <x:v>미정</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>필요 원자료</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
         <x:v>같은 run의 grid/step/order/mask/source identity와 오차 근거</x:v>
       </x:c>
-      <x:c r="H36" s="3" t="str">
-        <x:v>미정/미결속</x:v>
+      <x:c r="H39" s="3" t="str">
+        <x:v>미확보/미결속</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E36">
+  <x:conditionalFormatting sqref="E2:E39">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="미정"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R947b82125f244196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0996771391124366"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>